<commit_message>
added design project images
</commit_message>
<xml_diff>
--- a/portfolio_media/VEX_Volunteering.xlsx
+++ b/portfolio_media/VEX_Volunteering.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab1e07f38fe66cc6/Documents/Career/Website/test_v1/portfolio_generator/portfolio_media/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab1e07f38fe66cc6/Documents/Career/Website/rohanbpatel.github.io/portfolio_media/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="8_{2A76A078-DDA7-43B6-AA10-B3B492C6F618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F71FF97-7433-46A2-B29A-B13615E6C8C7}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="8_{2A76A078-DDA7-43B6-AA10-B3B492C6F618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B57162F-5CF5-4E01-8CEE-9E89A5446934}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="23226" windowHeight="13866" xr2:uid="{8903A9D0-2156-4902-9F33-57AFB774C556}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="40">
   <si>
     <t>https://www.robotevents.com/robot-competitions/vex-robotics-competition/RE-V5RC-24-7273.html#general-info</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>https://www.robotevents.com/robot-competitions/vex-iq-competition/RE-VIQC-21-5137.html#general-info</t>
+  </si>
+  <si>
+    <t>https://www.robotevents.com/robot-competitions/vex-robotics-competition/RE-V5RC-25-9947.html#general-info</t>
   </si>
 </sst>
 </file>
@@ -528,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27EF56ED-11A2-47F1-8507-03A24103749B}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="60.64453125" customWidth="1"/>
@@ -556,13 +559,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
       </c>
       <c r="C2" s="2">
-        <v>45982</v>
+        <v>46027</v>
       </c>
       <c r="D2" t="s">
         <v>20</v>
@@ -573,33 +576,33 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C3" s="2">
-        <v>45976</v>
+        <v>45982</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C4" s="2">
-        <v>45724</v>
+        <v>45976</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
         <v>32</v>
@@ -607,13 +610,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C5" s="2">
-        <v>45675</v>
+        <v>45724</v>
       </c>
       <c r="D5" t="s">
         <v>19</v>
@@ -624,16 +627,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C6" s="2">
-        <v>45660</v>
+        <v>45675</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s">
         <v>32</v>
@@ -641,16 +644,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2">
-        <v>45633</v>
+        <v>45660</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
         <v>32</v>
@@ -658,47 +661,47 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="C8" s="2">
-        <v>45618</v>
+        <v>45633</v>
       </c>
       <c r="D8" t="s">
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C9" s="2">
-        <v>45346</v>
+        <v>45618</v>
       </c>
       <c r="D9" t="s">
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C10" s="2">
-        <v>45311</v>
+        <v>45346</v>
       </c>
       <c r="D10" t="s">
         <v>19</v>
@@ -709,16 +712,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C11" s="2">
-        <v>45275</v>
+        <v>45311</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="E11" t="s">
         <v>32</v>
@@ -726,16 +729,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C12" s="2">
-        <v>45262</v>
+        <v>45275</v>
       </c>
       <c r="D12" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="E12" t="s">
         <v>32</v>
@@ -743,19 +746,19 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2">
-        <v>44898</v>
+        <v>45262</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.5">
@@ -763,27 +766,27 @@
         <v>28</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2">
-        <v>44534</v>
+        <v>44898</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="C15" s="2">
-        <v>44282</v>
+        <v>44534</v>
       </c>
       <c r="D15" t="s">
         <v>19</v>
@@ -792,9 +795,26 @@
         <v>32</v>
       </c>
     </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="2">
+        <v>44282</v>
+      </c>
+      <c r="D16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E15">
-    <sortCondition descending="1" ref="C15"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:E16">
+    <sortCondition descending="1" ref="C16"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
change robotevents to events.vex
</commit_message>
<xml_diff>
--- a/portfolio_media/VEX_Volunteering.xlsx
+++ b/portfolio_media/VEX_Volunteering.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohan\OneDrive\Documents\Career\Website\rohanbpatel.github.io\portfolio_media\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab1e07f38fe66cc6/Documents/Career/Website/rohanbpatel.github.io/portfolio_media/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCA1787-7246-4168-BF0B-5D67BB6CCB65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="6_{0272641C-0182-4F05-A401-33AAD6F775DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13093AF6-125B-4F3B-B917-E1CDB4926722}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" xr2:uid="{8903A9D0-2156-4902-9F33-57AFB774C556}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="23226" windowHeight="13866" xr2:uid="{8903A9D0-2156-4902-9F33-57AFB774C556}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -535,15 +535,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27EF56ED-11A2-47F1-8507-03A24103749B}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="60.62890625" customWidth="1"/>
-    <col min="2" max="2" width="42.9453125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.05078125" customWidth="1"/>
-    <col min="4" max="4" width="20.734375" customWidth="1"/>
+    <col min="1" max="1" width="60.64453125" customWidth="1"/>
+    <col min="2" max="2" width="42.9375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.05859375" customWidth="1"/>
+    <col min="4" max="4" width="20.703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -560,7 +560,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -577,7 +577,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -594,7 +594,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -611,7 +611,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -628,7 +628,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -645,7 +645,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -662,7 +662,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -679,7 +679,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -696,7 +696,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -713,7 +713,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -730,7 +730,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -747,7 +747,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -764,7 +764,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -781,7 +781,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -798,7 +798,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -815,7 +815,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
         <v>26</v>
       </c>

</xml_diff>